<commit_message>
docs: update design doc v1.3 - char limits, date validation, UI improvements
</commit_message>
<xml_diff>
--- a/docs/FoodLog_機能設計書.xlsx
+++ b/docs/FoodLog_機能設計書.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\anson\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\foodlog\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{541620F8-4445-477D-9359-DD4C632987D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F4A55C6-1614-4CDC-9F57-7CB10D09A5C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="380" yWindow="380" windowWidth="38400" windowHeight="15370" activeTab="1" xr2:uid="{43674596-D67D-4266-A19C-F0D950C013CA}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="51420" windowHeight="21100" activeTab="1" xr2:uid="{43674596-D67D-4266-A19C-F0D950C013CA}"/>
   </bookViews>
   <sheets>
     <sheet name="システム概要" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="375" uniqueCount="255">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="387" uniqueCount="264">
   <si>
     <t>FoodLog 機能設計書</t>
   </si>
@@ -487,9 +487,6 @@
     <t>低</t>
   </si>
   <si>
-    <t>名前・カテゴリ・説明・写真を編集モーダルで更新</t>
-  </si>
-  <si>
     <t>R-04</t>
   </si>
   <si>
@@ -748,27 +745,9 @@
     <t>🎉 全残作業完了！</t>
   </si>
   <si>
-    <t>機能一覧（最新版 v1.2）</t>
-  </si>
-  <si>
-    <t>最終更新: 2026-08-30　全機能実装完了</t>
-  </si>
-  <si>
     <t>全レストランをレビュー件数+最新注文日付きで取得</t>
   </si>
   <si>
-    <t>名前・カテゴリ・説明・写真（D&amp;D対応）を登録</t>
-  </si>
-  <si>
-    <t>カード or 詳細ページから確認ダイアログ付きで削除</t>
-  </si>
-  <si>
-    <t>日付・注文内容(複数行)・感想(500字制限)・評価を登録</t>
-  </si>
-  <si>
-    <t>編集モーダルで既存レビューを更新</t>
-  </si>
-  <si>
     <t>クリック or D&amp;Dでアップロード</t>
   </si>
   <si>
@@ -787,28 +766,76 @@
     <t>編集・追加後ページリロード不要</t>
   </si>
   <si>
-    <t>モバイル・PC両対応レイアウト</t>
-  </si>
-  <si>
     <t>U-04</t>
   </si>
   <si>
     <t>Last Order表示</t>
   </si>
   <si>
-    <t>ホーム画面に最新注文日をyyyy/mm/dd形式で表示</t>
-  </si>
-  <si>
     <t>U-05</t>
   </si>
   <si>
     <t>テキストエリア最適化</t>
   </si>
   <si>
-    <t>注文欄(複数行)・感想欄(500字固定)のリサイズ無効化</t>
-  </si>
-  <si>
-    <t>バージョン: 1.2（最終版）　最終更新: 2026-08-30　全機能実装完了</t>
+    <t>機能一覧（最新版 v1.3）</t>
+  </si>
+  <si>
+    <t>最終更新: 2026-08-30</t>
+  </si>
+  <si>
+    <t>名前(50字)・カテゴリ(200字)・説明(200字textarea)・写真</t>
+  </si>
+  <si>
+    <t>名前(50字)・カテゴリ(200字)・説明(200字textarea)・写真を更新</t>
+  </si>
+  <si>
+    <t>確認ダイアログ付きで削除（CASCADE）</t>
+  </si>
+  <si>
+    <t>日付(未来日不可)・注文内容(200字textarea)・感想(500字固定)・評価</t>
+  </si>
+  <si>
+    <t>編集モーダルで更新（同じ文字制限適用）</t>
+  </si>
+  <si>
+    <t>モバイル・PC両対応</t>
+  </si>
+  <si>
+    <t>最新注文日をyyyy/mm/dd形式で表示</t>
+  </si>
+  <si>
+    <t>注文欄(複数行)・感想欄(500字固定)リサイズ無効</t>
+  </si>
+  <si>
+    <t>U-06</t>
+  </si>
+  <si>
+    <t>文字数カウンター</t>
+  </si>
+  <si>
+    <t>全テキスト入力欄にリアルタイム文字数表示（80%で黄色・100%で赤）</t>
+  </si>
+  <si>
+    <t>U-07</t>
+  </si>
+  <si>
+    <t>未来日入力禁止</t>
+  </si>
+  <si>
+    <t>日付入力欄で未来の日付を選択不可</t>
+  </si>
+  <si>
+    <t>U-08</t>
+  </si>
+  <si>
+    <t>アスタリスク削除</t>
+  </si>
+  <si>
+    <t>全ラベルから * を削除（入力は引き続きrequired）</t>
+  </si>
+  <si>
+    <t>バージョン: 1.3　最終更新: 2026-08-30</t>
   </si>
 </sst>
 </file>
@@ -1350,7 +1377,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
-        <v>254</v>
+        <v>263</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="17" x14ac:dyDescent="0.4">
@@ -1478,7 +1505,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="19.5" x14ac:dyDescent="0.45">
       <c r="A1" s="18" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B1" s="18"/>
       <c r="C1" s="18"/>
@@ -1488,7 +1515,7 @@
     </row>
     <row r="2" spans="1:6" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A2" s="19" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B2" s="19"/>
       <c r="C2" s="19"/>
@@ -1499,7 +1526,7 @@
     <row r="3" spans="1:6" ht="14.5" x14ac:dyDescent="0.35"/>
     <row r="4" spans="1:6" ht="16" x14ac:dyDescent="0.4">
       <c r="A4" s="20" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B4" s="20"/>
       <c r="C4" s="20"/>
@@ -1509,59 +1536,59 @@
     </row>
     <row r="5" spans="1:6" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A5" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>162</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="C5" s="4" t="s">
         <v>163</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="D5" s="4" t="s">
         <v>164</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="E5" s="4" t="s">
         <v>165</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>166</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="58" x14ac:dyDescent="0.35">
       <c r="A6" s="14" t="s">
+        <v>166</v>
+      </c>
+      <c r="B6" s="14" t="s">
         <v>167</v>
-      </c>
-      <c r="B6" s="14" t="s">
-        <v>168</v>
       </c>
       <c r="C6" s="14" t="s">
         <v>5</v>
       </c>
       <c r="D6" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="E6" s="14" t="s">
         <v>169</v>
-      </c>
-      <c r="E6" s="14" t="s">
-        <v>170</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A7" s="15" t="s">
+        <v>170</v>
+      </c>
+      <c r="B7" s="15" t="s">
         <v>171</v>
       </c>
-      <c r="B7" s="15" t="s">
+      <c r="C7" s="15" t="s">
         <v>172</v>
       </c>
-      <c r="C7" s="15" t="s">
+      <c r="D7" s="15" t="s">
         <v>173</v>
       </c>
-      <c r="D7" s="15" t="s">
+      <c r="E7" s="15" t="s">
         <v>174</v>
-      </c>
-      <c r="E7" s="15" t="s">
-        <v>175</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="14.5" x14ac:dyDescent="0.35"/>
     <row r="9" spans="1:6" ht="16" x14ac:dyDescent="0.4">
       <c r="A9" s="20" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B9" s="20"/>
       <c r="C9" s="20"/>
@@ -1571,32 +1598,32 @@
     </row>
     <row r="10" spans="1:6" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A10" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="B10" s="4" t="s">
         <v>177</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="C10" s="4" t="s">
         <v>178</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>179</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A11" s="15" t="s">
+        <v>179</v>
+      </c>
+      <c r="B11" s="15" t="s">
         <v>180</v>
       </c>
-      <c r="B11" s="15" t="s">
+      <c r="C11" s="16" t="s">
         <v>181</v>
-      </c>
-      <c r="C11" s="16" t="s">
-        <v>182</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A12" s="14" t="s">
+        <v>182</v>
+      </c>
+      <c r="B12" s="14" t="s">
         <v>183</v>
-      </c>
-      <c r="B12" s="14" t="s">
-        <v>184</v>
       </c>
       <c r="C12" s="17" t="s">
         <v>72</v>
@@ -1604,10 +1631,10 @@
     </row>
     <row r="13" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A13" s="15" t="s">
+        <v>184</v>
+      </c>
+      <c r="B13" s="15" t="s">
         <v>185</v>
-      </c>
-      <c r="B13" s="15" t="s">
-        <v>186</v>
       </c>
       <c r="C13" s="16" t="s">
         <v>72</v>
@@ -1615,21 +1642,21 @@
     </row>
     <row r="14" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A14" s="14" t="s">
+        <v>186</v>
+      </c>
+      <c r="B14" s="14" t="s">
         <v>187</v>
       </c>
-      <c r="B14" s="14" t="s">
-        <v>188</v>
-      </c>
       <c r="C14" s="17" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A15" s="15" t="s">
+        <v>188</v>
+      </c>
+      <c r="B15" s="15" t="s">
         <v>189</v>
-      </c>
-      <c r="B15" s="15" t="s">
-        <v>190</v>
       </c>
       <c r="C15" s="16" t="s">
         <v>75</v>
@@ -1637,10 +1664,10 @@
     </row>
     <row r="16" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A16" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="B16" s="14" t="s">
         <v>191</v>
-      </c>
-      <c r="B16" s="14" t="s">
-        <v>192</v>
       </c>
       <c r="C16" s="17" t="s">
         <v>75</v>
@@ -1648,19 +1675,19 @@
     </row>
     <row r="17" spans="1:6" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A17" s="15" t="s">
+        <v>192</v>
+      </c>
+      <c r="B17" s="15" t="s">
         <v>193</v>
       </c>
-      <c r="B17" s="15" t="s">
-        <v>194</v>
-      </c>
       <c r="C17" s="16" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="14.5" x14ac:dyDescent="0.35"/>
     <row r="19" spans="1:6" ht="16" x14ac:dyDescent="0.4">
       <c r="A19" s="20" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B19" s="20"/>
       <c r="C19" s="20"/>
@@ -1670,32 +1697,32 @@
     </row>
     <row r="20" spans="1:6" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A20" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="B20" s="4" t="s">
         <v>177</v>
       </c>
-      <c r="B20" s="4" t="s">
+      <c r="C20" s="4" t="s">
         <v>178</v>
-      </c>
-      <c r="C20" s="4" t="s">
-        <v>179</v>
       </c>
     </row>
     <row r="21" spans="1:6" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A21" s="15" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B21" s="15" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C21" s="16" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="22" spans="1:6" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A22" s="14" t="s">
+        <v>196</v>
+      </c>
+      <c r="B22" s="14" t="s">
         <v>197</v>
-      </c>
-      <c r="B22" s="14" t="s">
-        <v>198</v>
       </c>
       <c r="C22" s="17" t="s">
         <v>95</v>
@@ -1703,10 +1730,10 @@
     </row>
     <row r="23" spans="1:6" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A23" s="15" t="s">
+        <v>198</v>
+      </c>
+      <c r="B23" s="15" t="s">
         <v>199</v>
-      </c>
-      <c r="B23" s="15" t="s">
-        <v>200</v>
       </c>
       <c r="C23" s="16" t="s">
         <v>72</v>
@@ -1714,10 +1741,10 @@
     </row>
     <row r="24" spans="1:6" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A24" s="14" t="s">
+        <v>200</v>
+      </c>
+      <c r="B24" s="14" t="s">
         <v>201</v>
-      </c>
-      <c r="B24" s="14" t="s">
-        <v>202</v>
       </c>
       <c r="C24" s="17" t="s">
         <v>77</v>
@@ -1725,32 +1752,32 @@
     </row>
     <row r="25" spans="1:6" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A25" s="15" t="s">
+        <v>202</v>
+      </c>
+      <c r="B25" s="15" t="s">
         <v>203</v>
       </c>
-      <c r="B25" s="15" t="s">
-        <v>204</v>
-      </c>
       <c r="C25" s="16" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="26" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A26" s="14" t="s">
+        <v>204</v>
+      </c>
+      <c r="B26" s="14" t="s">
         <v>205</v>
       </c>
-      <c r="B26" s="14" t="s">
+      <c r="C26" s="17" t="s">
         <v>206</v>
-      </c>
-      <c r="C26" s="17" t="s">
-        <v>207</v>
       </c>
     </row>
     <row r="27" spans="1:6" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A27" s="15" t="s">
+        <v>207</v>
+      </c>
+      <c r="B27" s="15" t="s">
         <v>208</v>
-      </c>
-      <c r="B27" s="15" t="s">
-        <v>209</v>
       </c>
       <c r="C27" s="16" t="s">
         <v>83</v>
@@ -1758,21 +1785,21 @@
     </row>
     <row r="28" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A28" s="14" t="s">
+        <v>209</v>
+      </c>
+      <c r="B28" s="14" t="s">
         <v>210</v>
       </c>
-      <c r="B28" s="14" t="s">
+      <c r="C28" s="17" t="s">
         <v>211</v>
-      </c>
-      <c r="C28" s="17" t="s">
-        <v>212</v>
       </c>
     </row>
     <row r="29" spans="1:6" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A29" s="15" t="s">
+        <v>212</v>
+      </c>
+      <c r="B29" s="15" t="s">
         <v>213</v>
-      </c>
-      <c r="B29" s="15" t="s">
-        <v>214</v>
       </c>
       <c r="C29" s="16" t="s">
         <v>88</v>
@@ -1780,10 +1807,10 @@
     </row>
     <row r="30" spans="1:6" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A30" s="14" t="s">
+        <v>214</v>
+      </c>
+      <c r="B30" s="14" t="s">
         <v>215</v>
-      </c>
-      <c r="B30" s="14" t="s">
-        <v>216</v>
       </c>
       <c r="C30" s="17" t="s">
         <v>85</v>
@@ -1791,13 +1818,13 @@
     </row>
     <row r="31" spans="1:6" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A31" s="15" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B31" s="15" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C31" s="16" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="32" spans="1:6" ht="14.5" x14ac:dyDescent="0.35"/>
@@ -2073,23 +2100,23 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1968643A-8311-4EAA-8541-885C9761494D}">
-  <dimension ref="A1:D31"/>
+  <dimension ref="A1:D34"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="35.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="31.08984375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="25.1796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="50.6328125" customWidth="1"/>
+    <col min="3" max="3" width="55.6328125" customWidth="1"/>
     <col min="4" max="4" width="20.6328125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="19.5" x14ac:dyDescent="0.45">
       <c r="A1" s="7" t="s">
-        <v>234</v>
+        <v>244</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
-        <v>235</v>
+        <v>245</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="16" x14ac:dyDescent="0.4">
@@ -2119,7 +2146,7 @@
         <v>73</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="D6" s="9" t="s">
         <v>74</v>
@@ -2133,7 +2160,7 @@
         <v>76</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>237</v>
+        <v>246</v>
       </c>
       <c r="D7" s="9" t="s">
         <v>74</v>
@@ -2147,7 +2174,7 @@
         <v>78</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>147</v>
+        <v>247</v>
       </c>
       <c r="D8" s="9" t="s">
         <v>74</v>
@@ -2155,13 +2182,13 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" s="6" t="s">
+        <v>147</v>
+      </c>
+      <c r="B9" s="6" t="s">
         <v>148</v>
       </c>
-      <c r="B9" s="6" t="s">
-        <v>149</v>
-      </c>
       <c r="C9" s="6" t="s">
-        <v>238</v>
+        <v>248</v>
       </c>
       <c r="D9" s="9" t="s">
         <v>74</v>
@@ -2208,7 +2235,7 @@
         <v>84</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>239</v>
+        <v>249</v>
       </c>
       <c r="D14" s="9" t="s">
         <v>74</v>
@@ -2236,7 +2263,7 @@
         <v>89</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>240</v>
+        <v>250</v>
       </c>
       <c r="D16" s="9" t="s">
         <v>74</v>
@@ -2269,7 +2296,7 @@
         <v>92</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>241</v>
+        <v>234</v>
       </c>
       <c r="D20" s="9" t="s">
         <v>74</v>
@@ -2283,7 +2310,7 @@
         <v>94</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>242</v>
+        <v>235</v>
       </c>
       <c r="D21" s="9" t="s">
         <v>74</v>
@@ -2297,7 +2324,7 @@
         <v>96</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>243</v>
+        <v>236</v>
       </c>
       <c r="D22" s="9" t="s">
         <v>74</v>
@@ -2305,13 +2332,13 @@
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="B23" s="6" t="s">
         <v>150</v>
       </c>
-      <c r="B23" s="6" t="s">
-        <v>151</v>
-      </c>
       <c r="C23" s="6" t="s">
-        <v>244</v>
+        <v>237</v>
       </c>
       <c r="D23" s="9" t="s">
         <v>74</v>
@@ -2319,7 +2346,7 @@
     </row>
     <row r="25" spans="1:4" ht="16" x14ac:dyDescent="0.4">
       <c r="A25" s="13" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.35">
@@ -2338,13 +2365,13 @@
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A27" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="B27" s="6" t="s">
         <v>153</v>
       </c>
-      <c r="B27" s="6" t="s">
-        <v>154</v>
-      </c>
       <c r="C27" s="6" t="s">
-        <v>245</v>
+        <v>238</v>
       </c>
       <c r="D27" s="9" t="s">
         <v>74</v>
@@ -2352,13 +2379,13 @@
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A28" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="B28" s="5" t="s">
         <v>155</v>
       </c>
-      <c r="B28" s="5" t="s">
-        <v>156</v>
-      </c>
       <c r="C28" s="5" t="s">
-        <v>246</v>
+        <v>239</v>
       </c>
       <c r="D28" s="9" t="s">
         <v>74</v>
@@ -2366,13 +2393,13 @@
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A29" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="B29" s="6" t="s">
         <v>157</v>
       </c>
-      <c r="B29" s="6" t="s">
-        <v>158</v>
-      </c>
       <c r="C29" s="6" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
       <c r="D29" s="9" t="s">
         <v>74</v>
@@ -2380,13 +2407,13 @@
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A30" s="5" t="s">
-        <v>248</v>
+        <v>240</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>249</v>
+        <v>241</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="D30" s="9" t="s">
         <v>74</v>
@@ -2394,15 +2421,57 @@
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A31" s="6" t="s">
-        <v>251</v>
+        <v>242</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>252</v>
+        <v>243</v>
       </c>
       <c r="C31" s="6" t="s">
         <v>253</v>
       </c>
       <c r="D31" s="9" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A32" s="5" t="s">
+        <v>254</v>
+      </c>
+      <c r="B32" s="5" t="s">
+        <v>255</v>
+      </c>
+      <c r="C32" s="5" t="s">
+        <v>256</v>
+      </c>
+      <c r="D32" s="9" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A33" s="6" t="s">
+        <v>257</v>
+      </c>
+      <c r="B33" s="6" t="s">
+        <v>258</v>
+      </c>
+      <c r="C33" s="6" t="s">
+        <v>259</v>
+      </c>
+      <c r="D33" s="9" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A34" s="5" t="s">
+        <v>260</v>
+      </c>
+      <c r="B34" s="5" t="s">
+        <v>261</v>
+      </c>
+      <c r="C34" s="5" t="s">
+        <v>262</v>
+      </c>
+      <c r="D34" s="9" t="s">
         <v>74</v>
       </c>
     </row>
@@ -2727,12 +2796,12 @@
   <sheetData>
     <row r="1" spans="1:6" ht="19.5" x14ac:dyDescent="0.45">
       <c r="A1" s="7" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
@@ -2749,10 +2818,10 @@
         <v>139</v>
       </c>
       <c r="E4" s="4" t="s">
+        <v>219</v>
+      </c>
+      <c r="F4" s="4" t="s">
         <v>220</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>221</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
@@ -2760,7 +2829,7 @@
         <v>1</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="C5" s="6" t="s">
         <v>140</v>
@@ -2772,7 +2841,7 @@
         <v>74</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
@@ -2780,7 +2849,7 @@
         <v>2</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C6" s="5" t="s">
         <v>140</v>
@@ -2792,7 +2861,7 @@
         <v>74</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
@@ -2800,7 +2869,7 @@
         <v>3</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C7" s="6" t="s">
         <v>143</v>
@@ -2812,7 +2881,7 @@
         <v>74</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.35">
@@ -2820,7 +2889,7 @@
         <v>4</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="C8" s="5" t="s">
         <v>143</v>
@@ -2832,7 +2901,7 @@
         <v>74</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.35">
@@ -2840,19 +2909,19 @@
         <v>5</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="C9" s="6" t="s">
         <v>146</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="E9" s="9" t="s">
         <v>74</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.35">
@@ -2860,24 +2929,24 @@
         <v>6</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="C10" s="5" t="s">
         <v>146</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="E10" s="9" t="s">
         <v>74</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" s="22" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B12" s="22"/>
       <c r="C12" s="22"/>

</xml_diff>

<commit_message>
feat: add restaurant address and review image upload; update design doc v1.4
</commit_message>
<xml_diff>
--- a/docs/FoodLog_機能設計書.xlsx
+++ b/docs/FoodLog_機能設計書.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\foodlog\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F4A55C6-1614-4CDC-9F57-7CB10D09A5C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A069BFF-F8C1-4574-90A8-E2595EC3E4EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="51420" windowHeight="21100" activeTab="1" xr2:uid="{43674596-D67D-4266-A19C-F0D950C013CA}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="387" uniqueCount="264">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="388" uniqueCount="265">
   <si>
     <t>FoodLog 機能設計書</t>
   </si>
@@ -292,9 +292,6 @@
     <t>レビュー一覧取得</t>
   </si>
   <si>
-    <t>特定レストランのレビューを新しい順で取得</t>
-  </si>
-  <si>
     <t>RV-02</t>
   </si>
   <si>
@@ -745,9 +742,6 @@
     <t>🎉 全残作業完了！</t>
   </si>
   <si>
-    <t>全レストランをレビュー件数+最新注文日付きで取得</t>
-  </si>
-  <si>
     <t>クリック or D&amp;Dでアップロード</t>
   </si>
   <si>
@@ -778,15 +772,9 @@
     <t>テキストエリア最適化</t>
   </si>
   <si>
-    <t>機能一覧（最新版 v1.3）</t>
-  </si>
-  <si>
     <t>最終更新: 2026-08-30</t>
   </si>
   <si>
-    <t>名前(50字)・カテゴリ(200字)・説明(200字textarea)・写真</t>
-  </si>
-  <si>
     <t>名前(50字)・カテゴリ(200字)・説明(200字textarea)・写真を更新</t>
   </si>
   <si>
@@ -835,7 +823,22 @@
     <t>全ラベルから * を削除（入力は引き続きrequired）</t>
   </si>
   <si>
-    <t>バージョン: 1.3　最終更新: 2026-08-30</t>
+    <t>機能一覧（最新版 v1.4）</t>
+  </si>
+  <si>
+    <t>名前(50字)・カテゴリ(200字)・説明(200字textarea)・住所(100字)・写真</t>
+  </si>
+  <si>
+    <t>名前(50字)・カテゴリ(200字)・説明(200字textarea)・住所(100字)・写真を更新</t>
+  </si>
+  <si>
+    <t>日付(未来日不可)・注文内容(200字)・感想(500字)・評価(必須)・写真(1枚)</t>
+  </si>
+  <si>
+    <t>編集モーダルで更新（画像変更対応・同じ文字制限適用）</t>
+  </si>
+  <si>
+    <t>バージョン: 1.4　最終更新: 2026-08-30</t>
   </si>
 </sst>
 </file>
@@ -1377,7 +1380,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="17" x14ac:dyDescent="0.4">
@@ -1505,7 +1508,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="19.5" x14ac:dyDescent="0.45">
       <c r="A1" s="18" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B1" s="18"/>
       <c r="C1" s="18"/>
@@ -1515,7 +1518,7 @@
     </row>
     <row r="2" spans="1:6" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A2" s="19" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B2" s="19"/>
       <c r="C2" s="19"/>
@@ -1526,7 +1529,7 @@
     <row r="3" spans="1:6" ht="14.5" x14ac:dyDescent="0.35"/>
     <row r="4" spans="1:6" ht="16" x14ac:dyDescent="0.4">
       <c r="A4" s="20" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B4" s="20"/>
       <c r="C4" s="20"/>
@@ -1536,59 +1539,59 @@
     </row>
     <row r="5" spans="1:6" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A5" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>161</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="C5" s="4" t="s">
         <v>162</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="D5" s="4" t="s">
         <v>163</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="E5" s="4" t="s">
         <v>164</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="58" x14ac:dyDescent="0.35">
       <c r="A6" s="14" t="s">
+        <v>165</v>
+      </c>
+      <c r="B6" s="14" t="s">
         <v>166</v>
-      </c>
-      <c r="B6" s="14" t="s">
-        <v>167</v>
       </c>
       <c r="C6" s="14" t="s">
         <v>5</v>
       </c>
       <c r="D6" s="14" t="s">
+        <v>167</v>
+      </c>
+      <c r="E6" s="14" t="s">
         <v>168</v>
-      </c>
-      <c r="E6" s="14" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A7" s="15" t="s">
+        <v>169</v>
+      </c>
+      <c r="B7" s="15" t="s">
         <v>170</v>
       </c>
-      <c r="B7" s="15" t="s">
+      <c r="C7" s="15" t="s">
         <v>171</v>
       </c>
-      <c r="C7" s="15" t="s">
+      <c r="D7" s="15" t="s">
         <v>172</v>
       </c>
-      <c r="D7" s="15" t="s">
+      <c r="E7" s="15" t="s">
         <v>173</v>
-      </c>
-      <c r="E7" s="15" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="14.5" x14ac:dyDescent="0.35"/>
     <row r="9" spans="1:6" ht="16" x14ac:dyDescent="0.4">
       <c r="A9" s="20" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B9" s="20"/>
       <c r="C9" s="20"/>
@@ -1598,32 +1601,32 @@
     </row>
     <row r="10" spans="1:6" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A10" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="B10" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="C10" s="4" t="s">
         <v>177</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>178</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A11" s="15" t="s">
+        <v>178</v>
+      </c>
+      <c r="B11" s="15" t="s">
         <v>179</v>
       </c>
-      <c r="B11" s="15" t="s">
+      <c r="C11" s="16" t="s">
         <v>180</v>
-      </c>
-      <c r="C11" s="16" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A12" s="14" t="s">
+        <v>181</v>
+      </c>
+      <c r="B12" s="14" t="s">
         <v>182</v>
-      </c>
-      <c r="B12" s="14" t="s">
-        <v>183</v>
       </c>
       <c r="C12" s="17" t="s">
         <v>72</v>
@@ -1631,10 +1634,10 @@
     </row>
     <row r="13" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A13" s="15" t="s">
+        <v>183</v>
+      </c>
+      <c r="B13" s="15" t="s">
         <v>184</v>
-      </c>
-      <c r="B13" s="15" t="s">
-        <v>185</v>
       </c>
       <c r="C13" s="16" t="s">
         <v>72</v>
@@ -1642,21 +1645,21 @@
     </row>
     <row r="14" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A14" s="14" t="s">
+        <v>185</v>
+      </c>
+      <c r="B14" s="14" t="s">
         <v>186</v>
       </c>
-      <c r="B14" s="14" t="s">
-        <v>187</v>
-      </c>
       <c r="C14" s="17" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A15" s="15" t="s">
+        <v>187</v>
+      </c>
+      <c r="B15" s="15" t="s">
         <v>188</v>
-      </c>
-      <c r="B15" s="15" t="s">
-        <v>189</v>
       </c>
       <c r="C15" s="16" t="s">
         <v>75</v>
@@ -1664,10 +1667,10 @@
     </row>
     <row r="16" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A16" s="14" t="s">
+        <v>189</v>
+      </c>
+      <c r="B16" s="14" t="s">
         <v>190</v>
-      </c>
-      <c r="B16" s="14" t="s">
-        <v>191</v>
       </c>
       <c r="C16" s="17" t="s">
         <v>75</v>
@@ -1675,19 +1678,19 @@
     </row>
     <row r="17" spans="1:6" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A17" s="15" t="s">
+        <v>191</v>
+      </c>
+      <c r="B17" s="15" t="s">
         <v>192</v>
       </c>
-      <c r="B17" s="15" t="s">
-        <v>193</v>
-      </c>
       <c r="C17" s="16" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="14.5" x14ac:dyDescent="0.35"/>
     <row r="19" spans="1:6" ht="16" x14ac:dyDescent="0.4">
       <c r="A19" s="20" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B19" s="20"/>
       <c r="C19" s="20"/>
@@ -1697,43 +1700,43 @@
     </row>
     <row r="20" spans="1:6" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A20" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="B20" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="B20" s="4" t="s">
+      <c r="C20" s="4" t="s">
         <v>177</v>
-      </c>
-      <c r="C20" s="4" t="s">
-        <v>178</v>
       </c>
     </row>
     <row r="21" spans="1:6" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A21" s="15" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B21" s="15" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C21" s="16" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="22" spans="1:6" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A22" s="14" t="s">
+        <v>195</v>
+      </c>
+      <c r="B22" s="14" t="s">
         <v>196</v>
       </c>
-      <c r="B22" s="14" t="s">
-        <v>197</v>
-      </c>
       <c r="C22" s="17" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A23" s="15" t="s">
+        <v>197</v>
+      </c>
+      <c r="B23" s="15" t="s">
         <v>198</v>
-      </c>
-      <c r="B23" s="15" t="s">
-        <v>199</v>
       </c>
       <c r="C23" s="16" t="s">
         <v>72</v>
@@ -1741,10 +1744,10 @@
     </row>
     <row r="24" spans="1:6" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A24" s="14" t="s">
+        <v>199</v>
+      </c>
+      <c r="B24" s="14" t="s">
         <v>200</v>
-      </c>
-      <c r="B24" s="14" t="s">
-        <v>201</v>
       </c>
       <c r="C24" s="17" t="s">
         <v>77</v>
@@ -1752,79 +1755,79 @@
     </row>
     <row r="25" spans="1:6" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A25" s="15" t="s">
+        <v>201</v>
+      </c>
+      <c r="B25" s="15" t="s">
         <v>202</v>
       </c>
-      <c r="B25" s="15" t="s">
-        <v>203</v>
-      </c>
       <c r="C25" s="16" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="26" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A26" s="14" t="s">
+        <v>203</v>
+      </c>
+      <c r="B26" s="14" t="s">
         <v>204</v>
       </c>
-      <c r="B26" s="14" t="s">
+      <c r="C26" s="17" t="s">
         <v>205</v>
-      </c>
-      <c r="C26" s="17" t="s">
-        <v>206</v>
       </c>
     </row>
     <row r="27" spans="1:6" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A27" s="15" t="s">
+        <v>206</v>
+      </c>
+      <c r="B27" s="15" t="s">
         <v>207</v>
       </c>
-      <c r="B27" s="15" t="s">
-        <v>208</v>
-      </c>
       <c r="C27" s="16" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A28" s="14" t="s">
+        <v>208</v>
+      </c>
+      <c r="B28" s="14" t="s">
         <v>209</v>
       </c>
-      <c r="B28" s="14" t="s">
+      <c r="C28" s="17" t="s">
         <v>210</v>
-      </c>
-      <c r="C28" s="17" t="s">
-        <v>211</v>
       </c>
     </row>
     <row r="29" spans="1:6" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A29" s="15" t="s">
+        <v>211</v>
+      </c>
+      <c r="B29" s="15" t="s">
         <v>212</v>
       </c>
-      <c r="B29" s="15" t="s">
-        <v>213</v>
-      </c>
       <c r="C29" s="16" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="30" spans="1:6" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A30" s="14" t="s">
+        <v>213</v>
+      </c>
+      <c r="B30" s="14" t="s">
         <v>214</v>
       </c>
-      <c r="B30" s="14" t="s">
-        <v>215</v>
-      </c>
       <c r="C30" s="17" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="31" spans="1:6" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A31" s="15" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B31" s="15" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C31" s="16" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="32" spans="1:6" ht="14.5" x14ac:dyDescent="0.35"/>
@@ -2111,12 +2114,12 @@
   <sheetData>
     <row r="1" spans="1:4" ht="19.5" x14ac:dyDescent="0.45">
       <c r="A1" s="7" t="s">
-        <v>244</v>
+        <v>259</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="16" x14ac:dyDescent="0.4">
@@ -2146,7 +2149,7 @@
         <v>73</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>233</v>
+        <v>260</v>
       </c>
       <c r="D6" s="9" t="s">
         <v>74</v>
@@ -2160,7 +2163,7 @@
         <v>76</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>246</v>
+        <v>261</v>
       </c>
       <c r="D7" s="9" t="s">
         <v>74</v>
@@ -2174,7 +2177,7 @@
         <v>78</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>247</v>
+        <v>243</v>
       </c>
       <c r="D8" s="9" t="s">
         <v>74</v>
@@ -2182,13 +2185,13 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" s="6" t="s">
+        <v>146</v>
+      </c>
+      <c r="B9" s="6" t="s">
         <v>147</v>
       </c>
-      <c r="B9" s="6" t="s">
-        <v>148</v>
-      </c>
       <c r="C9" s="6" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
       <c r="D9" s="9" t="s">
         <v>74</v>
@@ -2198,6 +2201,9 @@
       <c r="A11" s="13" t="s">
         <v>79</v>
       </c>
+      <c r="C11" t="s">
+        <v>262</v>
+      </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" s="4" t="s">
@@ -2221,7 +2227,7 @@
         <v>81</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>82</v>
+        <v>263</v>
       </c>
       <c r="D13" s="9" t="s">
         <v>74</v>
@@ -2229,13 +2235,13 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="B14" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="B14" s="5" t="s">
-        <v>84</v>
-      </c>
       <c r="C14" s="5" t="s">
-        <v>249</v>
+        <v>245</v>
       </c>
       <c r="D14" s="9" t="s">
         <v>74</v>
@@ -2243,13 +2249,13 @@
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="B15" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="B15" s="6" t="s">
+      <c r="C15" s="6" t="s">
         <v>86</v>
-      </c>
-      <c r="C15" s="6" t="s">
-        <v>87</v>
       </c>
       <c r="D15" s="9" t="s">
         <v>74</v>
@@ -2257,13 +2263,13 @@
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="B16" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="B16" s="5" t="s">
-        <v>89</v>
-      </c>
       <c r="C16" s="5" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
       <c r="D16" s="9" t="s">
         <v>74</v>
@@ -2271,7 +2277,7 @@
     </row>
     <row r="18" spans="1:4" ht="16" x14ac:dyDescent="0.4">
       <c r="A18" s="13" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.35">
@@ -2290,13 +2296,13 @@
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="B20" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="B20" s="5" t="s">
-        <v>92</v>
-      </c>
       <c r="C20" s="5" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="D20" s="9" t="s">
         <v>74</v>
@@ -2304,13 +2310,13 @@
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="B21" s="6" t="s">
         <v>93</v>
       </c>
-      <c r="B21" s="6" t="s">
-        <v>94</v>
-      </c>
       <c r="C21" s="6" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="D21" s="9" t="s">
         <v>74</v>
@@ -2318,13 +2324,13 @@
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="B22" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="B22" s="5" t="s">
-        <v>96</v>
-      </c>
       <c r="C22" s="5" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="D22" s="9" t="s">
         <v>74</v>
@@ -2332,13 +2338,13 @@
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="B23" s="6" t="s">
         <v>149</v>
       </c>
-      <c r="B23" s="6" t="s">
-        <v>150</v>
-      </c>
       <c r="C23" s="6" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="D23" s="9" t="s">
         <v>74</v>
@@ -2346,7 +2352,7 @@
     </row>
     <row r="25" spans="1:4" ht="16" x14ac:dyDescent="0.4">
       <c r="A25" s="13" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.35">
@@ -2365,13 +2371,13 @@
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A27" s="6" t="s">
+        <v>151</v>
+      </c>
+      <c r="B27" s="6" t="s">
         <v>152</v>
       </c>
-      <c r="B27" s="6" t="s">
-        <v>153</v>
-      </c>
       <c r="C27" s="6" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="D27" s="9" t="s">
         <v>74</v>
@@ -2379,13 +2385,13 @@
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A28" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="B28" s="5" t="s">
         <v>154</v>
       </c>
-      <c r="B28" s="5" t="s">
-        <v>155</v>
-      </c>
       <c r="C28" s="5" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="D28" s="9" t="s">
         <v>74</v>
@@ -2393,13 +2399,13 @@
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A29" s="6" t="s">
+        <v>155</v>
+      </c>
+      <c r="B29" s="6" t="s">
         <v>156</v>
       </c>
-      <c r="B29" s="6" t="s">
-        <v>157</v>
-      </c>
       <c r="C29" s="6" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
       <c r="D29" s="9" t="s">
         <v>74</v>
@@ -2407,13 +2413,13 @@
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A30" s="5" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="D30" s="9" t="s">
         <v>74</v>
@@ -2421,13 +2427,13 @@
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A31" s="6" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="D31" s="9" t="s">
         <v>74</v>
@@ -2435,13 +2441,13 @@
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A32" s="5" t="s">
-        <v>254</v>
+        <v>250</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>255</v>
+        <v>251</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>256</v>
+        <v>252</v>
       </c>
       <c r="D32" s="9" t="s">
         <v>74</v>
@@ -2449,13 +2455,13 @@
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A33" s="6" t="s">
-        <v>257</v>
+        <v>253</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>258</v>
+        <v>254</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>259</v>
+        <v>255</v>
       </c>
       <c r="D33" s="9" t="s">
         <v>74</v>
@@ -2463,13 +2469,13 @@
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A34" s="5" t="s">
-        <v>260</v>
+        <v>256</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>261</v>
+        <v>257</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="D34" s="9" t="s">
         <v>74</v>
@@ -2493,81 +2499,81 @@
   <sheetData>
     <row r="1" spans="1:4" ht="19.5" x14ac:dyDescent="0.45">
       <c r="A1" s="7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="16" x14ac:dyDescent="0.4">
       <c r="A3" s="8" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="B4" s="4" t="s">
         <v>99</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>100</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>27</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="B5" s="6" t="s">
         <v>102</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="C5" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="D5" s="6" t="s">
         <v>104</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="B6" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="C6" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="D6" s="5" t="s">
         <v>108</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B7" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="C7" s="6" t="s">
         <v>110</v>
       </c>
-      <c r="C7" s="6" t="s">
-        <v>111</v>
-      </c>
       <c r="D7" s="6" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" s="10" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" s="11" t="s">
+        <v>112</v>
+      </c>
+      <c r="B10" s="11" t="s">
         <v>113</v>
-      </c>
-      <c r="B10" s="11" t="s">
-        <v>114</v>
       </c>
       <c r="C10" s="11" t="s">
         <v>25</v>
@@ -2581,10 +2587,10 @@
         <v>32</v>
       </c>
       <c r="B11" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="C11" s="6" t="s">
         <v>115</v>
-      </c>
-      <c r="C11" s="6" t="s">
-        <v>116</v>
       </c>
       <c r="D11" s="6" t="s">
         <v>35</v>
@@ -2595,13 +2601,13 @@
         <v>36</v>
       </c>
       <c r="B12" s="12" t="s">
+        <v>114</v>
+      </c>
+      <c r="C12" s="12" t="s">
         <v>115</v>
       </c>
-      <c r="C12" s="12" t="s">
+      <c r="D12" s="12" t="s">
         <v>116</v>
-      </c>
-      <c r="D12" s="12" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
@@ -2610,10 +2616,10 @@
       </c>
       <c r="B13" s="6"/>
       <c r="C13" s="6" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
@@ -2622,84 +2628,84 @@
       </c>
       <c r="B14" s="12"/>
       <c r="C14" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="D14" s="12" t="s">
         <v>119</v>
-      </c>
-      <c r="D14" s="12" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="16" x14ac:dyDescent="0.4">
       <c r="A16" s="8" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="B17" s="4" t="s">
         <v>99</v>
-      </c>
-      <c r="B17" s="4" t="s">
-        <v>100</v>
       </c>
       <c r="C17" s="4" t="s">
         <v>27</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" s="5" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B18" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="C18" s="5" t="s">
         <v>122</v>
       </c>
-      <c r="C18" s="5" t="s">
+      <c r="D18" s="5" t="s">
         <v>123</v>
-      </c>
-      <c r="D18" s="5" t="s">
-        <v>124</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" s="6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B19" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="C19" s="6" t="s">
         <v>125</v>
       </c>
-      <c r="C19" s="6" t="s">
+      <c r="D19" s="6" t="s">
         <v>126</v>
-      </c>
-      <c r="D19" s="6" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="B20" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="B20" s="5" t="s">
+      <c r="C20" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="D20" s="5" t="s">
         <v>129</v>
-      </c>
-      <c r="C20" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="D20" s="5" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" s="10" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" s="11" t="s">
+        <v>112</v>
+      </c>
+      <c r="B23" s="11" t="s">
         <v>113</v>
-      </c>
-      <c r="B23" s="11" t="s">
-        <v>114</v>
       </c>
       <c r="C23" s="11" t="s">
         <v>25</v>
@@ -2713,10 +2719,10 @@
         <v>53</v>
       </c>
       <c r="B24" s="12" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C24" s="12" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D24" s="12" t="s">
         <v>31</v>
@@ -2727,10 +2733,10 @@
         <v>56</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D25" s="6" t="s">
         <v>58</v>
@@ -2741,10 +2747,10 @@
         <v>59</v>
       </c>
       <c r="B26" s="12" t="s">
+        <v>114</v>
+      </c>
+      <c r="C26" s="12" t="s">
         <v>115</v>
-      </c>
-      <c r="C26" s="12" t="s">
-        <v>116</v>
       </c>
       <c r="D26" s="12" t="s">
         <v>60</v>
@@ -2755,13 +2761,13 @@
         <v>61</v>
       </c>
       <c r="B27" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="C27" s="6" t="s">
         <v>115</v>
       </c>
-      <c r="C27" s="6" t="s">
-        <v>116</v>
-      </c>
       <c r="D27" s="6" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.35">
@@ -2770,10 +2776,10 @@
       </c>
       <c r="B28" s="12"/>
       <c r="C28" s="12" t="s">
+        <v>134</v>
+      </c>
+      <c r="D28" s="12" t="s">
         <v>135</v>
-      </c>
-      <c r="D28" s="12" t="s">
-        <v>136</v>
       </c>
     </row>
   </sheetData>
@@ -2796,32 +2802,32 @@
   <sheetData>
     <row r="1" spans="1:6" ht="19.5" x14ac:dyDescent="0.45">
       <c r="A1" s="7" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" s="4" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>3</v>
       </c>
       <c r="C4" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="D4" s="4" t="s">
         <v>138</v>
       </c>
-      <c r="D4" s="4" t="s">
-        <v>139</v>
-      </c>
       <c r="E4" s="4" t="s">
+        <v>218</v>
+      </c>
+      <c r="F4" s="4" t="s">
         <v>219</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>220</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
@@ -2829,19 +2835,19 @@
         <v>1</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C5" s="6" t="s">
+        <v>139</v>
+      </c>
+      <c r="D5" s="6" t="s">
         <v>140</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>141</v>
       </c>
       <c r="E5" s="9" t="s">
         <v>74</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
@@ -2849,19 +2855,19 @@
         <v>2</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E6" s="9" t="s">
         <v>74</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
@@ -2869,19 +2875,19 @@
         <v>3</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C7" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="D7" s="6" t="s">
         <v>143</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>144</v>
       </c>
       <c r="E7" s="9" t="s">
         <v>74</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.35">
@@ -2889,19 +2895,19 @@
         <v>4</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E8" s="9" t="s">
         <v>74</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.35">
@@ -2909,19 +2915,19 @@
         <v>5</v>
       </c>
       <c r="B9" s="6" t="s">
+        <v>226</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>145</v>
+      </c>
+      <c r="D9" s="6" t="s">
         <v>227</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>146</v>
-      </c>
-      <c r="D9" s="6" t="s">
-        <v>228</v>
       </c>
       <c r="E9" s="9" t="s">
         <v>74</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.35">
@@ -2929,24 +2935,24 @@
         <v>6</v>
       </c>
       <c r="B10" s="5" t="s">
+        <v>229</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="D10" s="5" t="s">
         <v>230</v>
-      </c>
-      <c r="C10" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>231</v>
       </c>
       <c r="E10" s="9" t="s">
         <v>74</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" s="22" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B12" s="22"/>
       <c r="C12" s="22"/>

</xml_diff>

<commit_message>
docs: update DB schema and R-03 description in Excel document
</commit_message>
<xml_diff>
--- a/docs/FoodLog_機能設計書.xlsx
+++ b/docs/FoodLog_機能設計書.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\foodlog\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A069BFF-F8C1-4574-90A8-E2595EC3E4EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5548215-6257-4D83-B0FB-C337DC0FF6B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="51420" windowHeight="21100" activeTab="1" xr2:uid="{43674596-D67D-4266-A19C-F0D950C013CA}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="388" uniqueCount="265">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="400" uniqueCount="268">
   <si>
     <t>FoodLog 機能設計書</t>
   </si>
@@ -112,12 +112,6 @@
     <t>http://localhost/foodlog/ でアプリ利用開始</t>
   </si>
   <si>
-    <t>DB設計</t>
-  </si>
-  <si>
-    <t>■ テーブル: restaurants</t>
-  </si>
-  <si>
     <t>カラム名</t>
   </si>
   <si>
@@ -160,33 +154,21 @@
     <t>VARCHAR(100)</t>
   </si>
   <si>
-    <t>料理カテゴリ（例: Japanese）</t>
-  </si>
-  <si>
     <t>description</t>
   </si>
   <si>
     <t>TEXT</t>
   </si>
   <si>
-    <t>短い説明文</t>
-  </si>
-  <si>
     <t>image</t>
   </si>
   <si>
-    <t>画像の相対パス（例: assets/images/ramen.png）</t>
-  </si>
-  <si>
     <t>emoji</t>
   </si>
   <si>
     <t>VARCHAR(10)</t>
   </si>
   <si>
-    <t>絵文字アイコン（旧仕様・現在未使用）</t>
-  </si>
-  <si>
     <t>created_at</t>
   </si>
   <si>
@@ -199,18 +181,12 @@
     <t>登録日時</t>
   </si>
   <si>
-    <t>■ テーブル: reviews</t>
-  </si>
-  <si>
     <t>レビューID</t>
   </si>
   <si>
     <t>restaurant_id</t>
   </si>
   <si>
-    <t>NOT NULL, FK → restaurants.id</t>
-  </si>
-  <si>
     <t>対象レストランID</t>
   </si>
   <si>
@@ -232,24 +208,15 @@
     <t>impression</t>
   </si>
   <si>
-    <t>感想・インプレッション</t>
-  </si>
-  <si>
     <t>rating</t>
   </si>
   <si>
     <t>TINYINT</t>
   </si>
   <si>
-    <t>NULL可</t>
-  </si>
-  <si>
     <t>評価（1〜5）</t>
   </si>
   <si>
-    <t>※ restaurant_id は restaurants.id を参照。レストラン削除時にレビューも CASCADE削除。</t>
-  </si>
-  <si>
     <t>■ レストラン管理</t>
   </si>
   <si>
@@ -839,13 +806,55 @@
   </si>
   <si>
     <t>バージョン: 1.4　最終更新: 2026-08-30</t>
+  </si>
+  <si>
+    <t>DB設計（最新版 v1.4）</t>
+  </si>
+  <si>
+    <t>restaurants (レストラン情報)</t>
+  </si>
+  <si>
+    <t>データ型</t>
+  </si>
+  <si>
+    <t>論理名</t>
+  </si>
+  <si>
+    <t>店名</t>
+  </si>
+  <si>
+    <t>NULL</t>
+  </si>
+  <si>
+    <t>カテゴリ（Japanese, Italian等）</t>
+  </si>
+  <si>
+    <t>説明・紹介文</t>
+  </si>
+  <si>
+    <t>address</t>
+  </si>
+  <si>
+    <t>住所</t>
+  </si>
+  <si>
+    <t>画像ファイルのパス</t>
+  </si>
+  <si>
+    <t>デフォルト絵文字（シードデータ用）</t>
+  </si>
+  <si>
+    <t>reviews (レビュー情報)</t>
+  </si>
+  <si>
+    <t>FK (restaurants.id) ON DELETE CASCADE</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -902,13 +911,6 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF00607F"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
       <color rgb="FF235637"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -946,7 +948,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -968,12 +970,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFFF"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFCCF2FF"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1002,7 +998,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1012,24 +1008,23 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1380,7 +1375,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
-        <v>264</v>
+        <v>253</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="17" x14ac:dyDescent="0.4">
@@ -1508,7 +1503,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="19.5" x14ac:dyDescent="0.45">
       <c r="A1" s="18" t="s">
-        <v>157</v>
+        <v>146</v>
       </c>
       <c r="B1" s="18"/>
       <c r="C1" s="18"/>
@@ -1518,7 +1513,7 @@
     </row>
     <row r="2" spans="1:6" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A2" s="19" t="s">
-        <v>158</v>
+        <v>147</v>
       </c>
       <c r="B2" s="19"/>
       <c r="C2" s="19"/>
@@ -1529,7 +1524,7 @@
     <row r="3" spans="1:6" ht="14.5" x14ac:dyDescent="0.35"/>
     <row r="4" spans="1:6" ht="16" x14ac:dyDescent="0.4">
       <c r="A4" s="20" t="s">
-        <v>159</v>
+        <v>148</v>
       </c>
       <c r="B4" s="20"/>
       <c r="C4" s="20"/>
@@ -1539,59 +1534,59 @@
     </row>
     <row r="5" spans="1:6" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A5" s="4" t="s">
-        <v>160</v>
+        <v>149</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>162</v>
+        <v>151</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>163</v>
+        <v>152</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>164</v>
+        <v>153</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="58" x14ac:dyDescent="0.35">
       <c r="A6" s="14" t="s">
-        <v>165</v>
+        <v>154</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>166</v>
+        <v>155</v>
       </c>
       <c r="C6" s="14" t="s">
         <v>5</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>167</v>
+        <v>156</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>168</v>
+        <v>157</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A7" s="15" t="s">
-        <v>169</v>
+        <v>158</v>
       </c>
       <c r="B7" s="15" t="s">
-        <v>170</v>
+        <v>159</v>
       </c>
       <c r="C7" s="15" t="s">
-        <v>171</v>
+        <v>160</v>
       </c>
       <c r="D7" s="15" t="s">
-        <v>172</v>
+        <v>161</v>
       </c>
       <c r="E7" s="15" t="s">
-        <v>173</v>
+        <v>162</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="14.5" x14ac:dyDescent="0.35"/>
     <row r="9" spans="1:6" ht="16" x14ac:dyDescent="0.4">
       <c r="A9" s="20" t="s">
-        <v>174</v>
+        <v>163</v>
       </c>
       <c r="B9" s="20"/>
       <c r="C9" s="20"/>
@@ -1601,96 +1596,96 @@
     </row>
     <row r="10" spans="1:6" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A10" s="4" t="s">
-        <v>175</v>
+        <v>164</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>176</v>
+        <v>165</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>177</v>
+        <v>166</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A11" s="15" t="s">
-        <v>178</v>
+        <v>167</v>
       </c>
       <c r="B11" s="15" t="s">
-        <v>179</v>
+        <v>168</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>180</v>
+        <v>169</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A12" s="14" t="s">
-        <v>181</v>
+        <v>170</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>182</v>
+        <v>171</v>
       </c>
       <c r="C12" s="17" t="s">
-        <v>72</v>
+        <v>61</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A13" s="15" t="s">
-        <v>183</v>
+        <v>172</v>
       </c>
       <c r="B13" s="15" t="s">
-        <v>184</v>
+        <v>173</v>
       </c>
       <c r="C13" s="16" t="s">
-        <v>72</v>
+        <v>61</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A14" s="14" t="s">
-        <v>185</v>
+        <v>174</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>186</v>
+        <v>175</v>
       </c>
       <c r="C14" s="17" t="s">
-        <v>146</v>
+        <v>135</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A15" s="15" t="s">
-        <v>187</v>
+        <v>176</v>
       </c>
       <c r="B15" s="15" t="s">
-        <v>188</v>
+        <v>177</v>
       </c>
       <c r="C15" s="16" t="s">
-        <v>75</v>
+        <v>64</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A16" s="14" t="s">
-        <v>189</v>
+        <v>178</v>
       </c>
       <c r="B16" s="14" t="s">
-        <v>190</v>
+        <v>179</v>
       </c>
       <c r="C16" s="17" t="s">
-        <v>75</v>
+        <v>64</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A17" s="15" t="s">
-        <v>191</v>
+        <v>180</v>
       </c>
       <c r="B17" s="15" t="s">
-        <v>192</v>
+        <v>181</v>
       </c>
       <c r="C17" s="16" t="s">
-        <v>180</v>
+        <v>169</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="14.5" x14ac:dyDescent="0.35"/>
     <row r="19" spans="1:6" ht="16" x14ac:dyDescent="0.4">
       <c r="A19" s="20" t="s">
-        <v>193</v>
+        <v>182</v>
       </c>
       <c r="B19" s="20"/>
       <c r="C19" s="20"/>
@@ -1700,134 +1695,134 @@
     </row>
     <row r="20" spans="1:6" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A20" s="4" t="s">
-        <v>175</v>
+        <v>164</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>176</v>
+        <v>165</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>177</v>
+        <v>166</v>
       </c>
     </row>
     <row r="21" spans="1:6" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A21" s="15" t="s">
-        <v>178</v>
+        <v>167</v>
       </c>
       <c r="B21" s="15" t="s">
-        <v>194</v>
+        <v>183</v>
       </c>
       <c r="C21" s="16" t="s">
-        <v>180</v>
+        <v>169</v>
       </c>
     </row>
     <row r="22" spans="1:6" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A22" s="14" t="s">
-        <v>195</v>
+        <v>184</v>
       </c>
       <c r="B22" s="14" t="s">
-        <v>196</v>
+        <v>185</v>
       </c>
       <c r="C22" s="17" t="s">
-        <v>94</v>
+        <v>83</v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A23" s="15" t="s">
-        <v>197</v>
+        <v>186</v>
       </c>
       <c r="B23" s="15" t="s">
-        <v>198</v>
+        <v>187</v>
       </c>
       <c r="C23" s="16" t="s">
-        <v>72</v>
+        <v>61</v>
       </c>
     </row>
     <row r="24" spans="1:6" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A24" s="14" t="s">
-        <v>199</v>
+        <v>188</v>
       </c>
       <c r="B24" s="14" t="s">
-        <v>200</v>
+        <v>189</v>
       </c>
       <c r="C24" s="17" t="s">
-        <v>77</v>
+        <v>66</v>
       </c>
     </row>
     <row r="25" spans="1:6" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A25" s="15" t="s">
-        <v>201</v>
+        <v>190</v>
       </c>
       <c r="B25" s="15" t="s">
-        <v>202</v>
+        <v>191</v>
       </c>
       <c r="C25" s="16" t="s">
-        <v>146</v>
+        <v>135</v>
       </c>
     </row>
     <row r="26" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A26" s="14" t="s">
-        <v>203</v>
+        <v>192</v>
       </c>
       <c r="B26" s="14" t="s">
-        <v>204</v>
+        <v>193</v>
       </c>
       <c r="C26" s="17" t="s">
-        <v>205</v>
+        <v>194</v>
       </c>
     </row>
     <row r="27" spans="1:6" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A27" s="15" t="s">
-        <v>206</v>
+        <v>195</v>
       </c>
       <c r="B27" s="15" t="s">
-        <v>207</v>
+        <v>196</v>
       </c>
       <c r="C27" s="16" t="s">
-        <v>82</v>
+        <v>71</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A28" s="14" t="s">
-        <v>208</v>
+        <v>197</v>
       </c>
       <c r="B28" s="14" t="s">
-        <v>209</v>
+        <v>198</v>
       </c>
       <c r="C28" s="17" t="s">
-        <v>210</v>
+        <v>199</v>
       </c>
     </row>
     <row r="29" spans="1:6" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A29" s="15" t="s">
-        <v>211</v>
+        <v>200</v>
       </c>
       <c r="B29" s="15" t="s">
-        <v>212</v>
+        <v>201</v>
       </c>
       <c r="C29" s="16" t="s">
-        <v>87</v>
+        <v>76</v>
       </c>
     </row>
     <row r="30" spans="1:6" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A30" s="14" t="s">
-        <v>213</v>
+        <v>202</v>
       </c>
       <c r="B30" s="14" t="s">
-        <v>214</v>
+        <v>203</v>
       </c>
       <c r="C30" s="17" t="s">
-        <v>84</v>
+        <v>73</v>
       </c>
     </row>
     <row r="31" spans="1:6" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A31" s="15" t="s">
-        <v>152</v>
+        <v>141</v>
       </c>
       <c r="B31" s="15" t="s">
-        <v>215</v>
+        <v>204</v>
       </c>
       <c r="C31" s="16" t="s">
-        <v>151</v>
+        <v>140</v>
       </c>
     </row>
     <row r="32" spans="1:6" ht="14.5" x14ac:dyDescent="0.35"/>
@@ -1845,258 +1840,288 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB947EF0-FA3F-4853-ABD1-0DF7DBC08E2E}">
-  <dimension ref="A1:D22"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="23" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="28.81640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.1796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="27.08984375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="45.6328125" customWidth="1"/>
+    <col min="3" max="3" width="35.6328125" customWidth="1"/>
+    <col min="4" max="4" width="30.6328125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="19.5" x14ac:dyDescent="0.45">
       <c r="A1" s="7" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" s="2" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="16" x14ac:dyDescent="0.4">
+      <c r="A4" s="13" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" s="4" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" ht="16" x14ac:dyDescent="0.4">
-      <c r="A3" s="8" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A4" s="4" t="s">
+      <c r="B5" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="C5" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="B4" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A5" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>31</v>
+      <c r="D5" s="4" t="s">
+        <v>257</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" s="5" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="6" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="C7" s="6"/>
+        <v>31</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>32</v>
+      </c>
       <c r="D7" s="6" t="s">
-        <v>38</v>
+        <v>258</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" s="5" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="C8" s="5"/>
+        <v>35</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>259</v>
+      </c>
       <c r="D8" s="5" t="s">
-        <v>41</v>
+        <v>260</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" s="6" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="C9" s="6"/>
+        <v>37</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>259</v>
+      </c>
       <c r="D9" s="6" t="s">
-        <v>43</v>
+        <v>261</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" s="5" t="s">
-        <v>44</v>
+        <v>262</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="C10" s="5"/>
+        <v>35</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>259</v>
+      </c>
       <c r="D10" s="5" t="s">
-        <v>46</v>
+        <v>263</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" s="6" t="s">
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>48</v>
+        <v>31</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>49</v>
+        <v>259</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" ht="16" x14ac:dyDescent="0.4">
-      <c r="A13" s="8" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A14" s="4" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>259</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="16" x14ac:dyDescent="0.4">
+      <c r="A15" s="13" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A16" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="C16" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="B14" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="D14" s="4" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A15" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="B15" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="C15" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="D15" s="6" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A16" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="B16" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="C16" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="D16" s="5" t="s">
-        <v>55</v>
+      <c r="D16" s="4" t="s">
+        <v>257</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" s="6" t="s">
-        <v>56</v>
+        <v>26</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>57</v>
+        <v>27</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>58</v>
+        <v>45</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" s="5" t="s">
-        <v>59</v>
+        <v>46</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>40</v>
+        <v>27</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>34</v>
+        <v>267</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>60</v>
+        <v>47</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" s="6" t="s">
-        <v>61</v>
+        <v>48</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>40</v>
+        <v>49</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>62</v>
+        <v>50</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" s="5" t="s">
-        <v>63</v>
+        <v>51</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>64</v>
+        <v>37</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>65</v>
+        <v>32</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>66</v>
+        <v>52</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21" s="6" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>48</v>
+        <v>37</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>49</v>
+        <v>32</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>50</v>
+        <v>122</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A22" s="21" t="s">
-        <v>67</v>
-      </c>
-      <c r="B22" s="21"/>
-      <c r="C22" s="21"/>
-      <c r="D22" s="21"/>
+      <c r="A22" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>259</v>
+      </c>
+      <c r="D22" s="5" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A23" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>259</v>
+      </c>
+      <c r="D23" s="6" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A24" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="C24" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="D24" s="5" t="s">
+        <v>44</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A22:D22"/>
-  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -2114,371 +2139,371 @@
   <sheetData>
     <row r="1" spans="1:4" ht="19.5" x14ac:dyDescent="0.45">
       <c r="A1" s="7" t="s">
-        <v>259</v>
+        <v>248</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
-        <v>242</v>
+        <v>231</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="16" x14ac:dyDescent="0.4">
       <c r="A4" s="13" t="s">
-        <v>68</v>
+        <v>57</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" s="4" t="s">
-        <v>69</v>
+        <v>58</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>70</v>
+        <v>59</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>71</v>
+        <v>60</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" s="5" t="s">
-        <v>72</v>
+        <v>61</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>73</v>
+        <v>62</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>260</v>
+        <v>249</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>74</v>
+        <v>63</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="6" t="s">
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>76</v>
+        <v>65</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>261</v>
+        <v>250</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>74</v>
+        <v>63</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" s="5" t="s">
-        <v>77</v>
+        <v>66</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>243</v>
+        <v>232</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>74</v>
+        <v>63</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" s="6" t="s">
-        <v>146</v>
+        <v>135</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>147</v>
+        <v>136</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>244</v>
+        <v>233</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>74</v>
+        <v>63</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="16" x14ac:dyDescent="0.4">
       <c r="A11" s="13" t="s">
-        <v>79</v>
+        <v>68</v>
       </c>
       <c r="C11" t="s">
-        <v>262</v>
+        <v>251</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" s="4" t="s">
-        <v>69</v>
+        <v>58</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>70</v>
+        <v>59</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>71</v>
+        <v>60</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" s="6" t="s">
-        <v>80</v>
+        <v>69</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>81</v>
+        <v>70</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>263</v>
+        <v>252</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>74</v>
+        <v>63</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" s="5" t="s">
-        <v>82</v>
+        <v>71</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>83</v>
+        <v>72</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>245</v>
+        <v>234</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>74</v>
+        <v>63</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" s="6" t="s">
-        <v>84</v>
+        <v>73</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>85</v>
+        <v>74</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>86</v>
+        <v>75</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>74</v>
+        <v>63</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" s="5" t="s">
-        <v>87</v>
+        <v>76</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>246</v>
+        <v>235</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>74</v>
+        <v>63</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="16" x14ac:dyDescent="0.4">
       <c r="A18" s="13" t="s">
-        <v>89</v>
+        <v>78</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" s="4" t="s">
-        <v>69</v>
+        <v>58</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>70</v>
+        <v>59</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>71</v>
+        <v>60</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" s="5" t="s">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>232</v>
+        <v>221</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>74</v>
+        <v>63</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21" s="6" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>233</v>
+        <v>222</v>
       </c>
       <c r="D21" s="9" t="s">
-        <v>74</v>
+        <v>63</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" s="5" t="s">
-        <v>94</v>
+        <v>83</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>95</v>
+        <v>84</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>234</v>
+        <v>223</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>74</v>
+        <v>63</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" s="6" t="s">
-        <v>148</v>
+        <v>137</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>149</v>
+        <v>138</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>235</v>
+        <v>224</v>
       </c>
       <c r="D23" s="9" t="s">
-        <v>74</v>
+        <v>63</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="16" x14ac:dyDescent="0.4">
       <c r="A25" s="13" t="s">
-        <v>150</v>
+        <v>139</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A26" s="4" t="s">
-        <v>69</v>
+        <v>58</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>70</v>
+        <v>59</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>71</v>
+        <v>60</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A27" s="6" t="s">
-        <v>151</v>
+        <v>140</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>152</v>
+        <v>141</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>236</v>
+        <v>225</v>
       </c>
       <c r="D27" s="9" t="s">
-        <v>74</v>
+        <v>63</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A28" s="5" t="s">
-        <v>153</v>
+        <v>142</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>154</v>
+        <v>143</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>237</v>
+        <v>226</v>
       </c>
       <c r="D28" s="9" t="s">
-        <v>74</v>
+        <v>63</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A29" s="6" t="s">
-        <v>155</v>
+        <v>144</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>247</v>
+        <v>236</v>
       </c>
       <c r="D29" s="9" t="s">
-        <v>74</v>
+        <v>63</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A30" s="5" t="s">
-        <v>238</v>
+        <v>227</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>248</v>
+        <v>237</v>
       </c>
       <c r="D30" s="9" t="s">
-        <v>74</v>
+        <v>63</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A31" s="6" t="s">
-        <v>240</v>
+        <v>229</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>241</v>
+        <v>230</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>249</v>
+        <v>238</v>
       </c>
       <c r="D31" s="9" t="s">
-        <v>74</v>
+        <v>63</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A32" s="5" t="s">
-        <v>250</v>
+        <v>239</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>251</v>
+        <v>240</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>252</v>
+        <v>241</v>
       </c>
       <c r="D32" s="9" t="s">
-        <v>74</v>
+        <v>63</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A33" s="6" t="s">
-        <v>253</v>
+        <v>242</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>254</v>
+        <v>243</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>255</v>
+        <v>244</v>
       </c>
       <c r="D33" s="9" t="s">
-        <v>74</v>
+        <v>63</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A34" s="5" t="s">
-        <v>256</v>
+        <v>245</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>257</v>
+        <v>246</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>258</v>
+        <v>247</v>
       </c>
       <c r="D34" s="9" t="s">
-        <v>74</v>
+        <v>63</v>
       </c>
     </row>
   </sheetData>
@@ -2499,287 +2524,287 @@
   <sheetData>
     <row r="1" spans="1:4" ht="19.5" x14ac:dyDescent="0.45">
       <c r="A1" s="7" t="s">
-        <v>96</v>
+        <v>85</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="16" x14ac:dyDescent="0.4">
       <c r="A3" s="8" t="s">
-        <v>97</v>
+        <v>86</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="4" t="s">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>99</v>
+        <v>88</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>100</v>
+        <v>89</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" s="6" t="s">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>103</v>
+        <v>92</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>104</v>
+        <v>93</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" s="5" t="s">
-        <v>105</v>
+        <v>94</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>107</v>
+        <v>96</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>108</v>
+        <v>97</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="6" t="s">
-        <v>105</v>
+        <v>94</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>109</v>
+        <v>98</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>110</v>
+        <v>99</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>108</v>
+        <v>97</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" s="10" t="s">
-        <v>111</v>
+        <v>100</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" s="11" t="s">
-        <v>112</v>
+        <v>101</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>113</v>
+        <v>102</v>
       </c>
       <c r="C10" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="D10" s="11" t="s">
         <v>25</v>
-      </c>
-      <c r="D10" s="11" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" s="6" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>114</v>
+        <v>103</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>115</v>
+        <v>104</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" s="12" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>114</v>
+        <v>103</v>
       </c>
       <c r="C12" s="12" t="s">
-        <v>115</v>
+        <v>104</v>
       </c>
       <c r="D12" s="12" t="s">
-        <v>116</v>
+        <v>105</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" s="6" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B13" s="6"/>
       <c r="C13" s="6" t="s">
-        <v>115</v>
+        <v>104</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>117</v>
+        <v>106</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" s="12" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="B14" s="12"/>
       <c r="C14" s="12" t="s">
-        <v>118</v>
+        <v>107</v>
       </c>
       <c r="D14" s="12" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="16" x14ac:dyDescent="0.4">
       <c r="A16" s="8" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" s="4" t="s">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>99</v>
+        <v>88</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>100</v>
+        <v>89</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" s="5" t="s">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>121</v>
+        <v>110</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>122</v>
+        <v>111</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>123</v>
+        <v>112</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" s="6" t="s">
-        <v>105</v>
+        <v>94</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>124</v>
+        <v>113</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>125</v>
+        <v>114</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>126</v>
+        <v>115</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" s="5" t="s">
-        <v>127</v>
+        <v>116</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>128</v>
+        <v>117</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>85</v>
+        <v>74</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>129</v>
+        <v>118</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" s="10" t="s">
-        <v>130</v>
+        <v>119</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" s="11" t="s">
-        <v>112</v>
+        <v>101</v>
       </c>
       <c r="B23" s="11" t="s">
-        <v>113</v>
+        <v>102</v>
       </c>
       <c r="C23" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="D23" s="11" t="s">
         <v>25</v>
-      </c>
-      <c r="D23" s="11" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A24" s="12" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="B24" s="12" t="s">
-        <v>114</v>
+        <v>103</v>
       </c>
       <c r="C24" s="12" t="s">
-        <v>131</v>
+        <v>120</v>
       </c>
       <c r="D24" s="12" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A25" s="6" t="s">
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>114</v>
+        <v>103</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>132</v>
+        <v>121</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A26" s="12" t="s">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="B26" s="12" t="s">
-        <v>114</v>
+        <v>103</v>
       </c>
       <c r="C26" s="12" t="s">
-        <v>115</v>
+        <v>104</v>
       </c>
       <c r="D26" s="12" t="s">
-        <v>60</v>
+        <v>52</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A27" s="6" t="s">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>114</v>
+        <v>103</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>115</v>
+        <v>104</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>133</v>
+        <v>122</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A28" s="12" t="s">
-        <v>63</v>
+        <v>54</v>
       </c>
       <c r="B28" s="12"/>
       <c r="C28" s="12" t="s">
-        <v>134</v>
+        <v>123</v>
       </c>
       <c r="D28" s="12" t="s">
-        <v>135</v>
+        <v>124</v>
       </c>
     </row>
   </sheetData>
@@ -2802,32 +2827,32 @@
   <sheetData>
     <row r="1" spans="1:6" ht="19.5" x14ac:dyDescent="0.45">
       <c r="A1" s="7" t="s">
-        <v>216</v>
+        <v>205</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
-        <v>217</v>
+        <v>206</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" s="4" t="s">
-        <v>136</v>
+        <v>125</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>3</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>137</v>
+        <v>126</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>138</v>
+        <v>127</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>218</v>
+        <v>207</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>219</v>
+        <v>208</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
@@ -2835,19 +2860,19 @@
         <v>1</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>220</v>
+        <v>209</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>139</v>
+        <v>128</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>140</v>
+        <v>129</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>74</v>
+        <v>63</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>221</v>
+        <v>210</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
@@ -2855,19 +2880,19 @@
         <v>2</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>222</v>
+        <v>211</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>139</v>
+        <v>128</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>141</v>
+        <v>130</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>74</v>
+        <v>63</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>221</v>
+        <v>210</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
@@ -2875,19 +2900,19 @@
         <v>3</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>223</v>
+        <v>212</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>142</v>
+        <v>131</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>143</v>
+        <v>132</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>74</v>
+        <v>63</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>224</v>
+        <v>213</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.35">
@@ -2895,19 +2920,19 @@
         <v>4</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>225</v>
+        <v>214</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>142</v>
+        <v>131</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>144</v>
+        <v>133</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>74</v>
+        <v>63</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>224</v>
+        <v>213</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.35">
@@ -2915,19 +2940,19 @@
         <v>5</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>226</v>
+        <v>215</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>145</v>
+        <v>134</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>227</v>
+        <v>216</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>74</v>
+        <v>63</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>228</v>
+        <v>217</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.35">
@@ -2935,30 +2960,30 @@
         <v>6</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>229</v>
+        <v>218</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>145</v>
+        <v>134</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>230</v>
+        <v>219</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>74</v>
+        <v>63</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>228</v>
+        <v>217</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A12" s="22" t="s">
-        <v>231</v>
-      </c>
-      <c r="B12" s="22"/>
-      <c r="C12" s="22"/>
-      <c r="D12" s="22"/>
-      <c r="E12" s="22"/>
-      <c r="F12" s="22"/>
+      <c r="A12" s="21" t="s">
+        <v>220</v>
+      </c>
+      <c r="B12" s="21"/>
+      <c r="C12" s="21"/>
+      <c r="D12" s="21"/>
+      <c r="E12" s="21"/>
+      <c r="F12" s="21"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>